<commit_message>
RIPTE real a precios del último mes con RIPTE e IPC
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012WiZx484kRcrrNZ4YGQ81g
</commit_message>
<xml_diff>
--- a/data/excel/ripte_real.xlsx
+++ b/data/excel/ripte_real.xlsx
@@ -438,7 +438,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>RIPTE real, a precios del último mes del IPC</t>
+          <t>RIPTE real, a precios del último mes disponible</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -460,7 +460,7 @@
         <v>20690.14</v>
       </c>
       <c r="C2" t="n">
-        <v>2589195.32033112</v>
+        <v>2540080.0728724</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
@@ -473,7 +473,7 @@
         <v>20719.61758472386</v>
       </c>
       <c r="C3" t="n">
-        <v>2592884.189735662</v>
+        <v>2543698.9669714</v>
       </c>
       <c r="D3" t="n">
         <v>0.1424716542462345</v>
@@ -488,7 +488,7 @@
         <v>20719.33599457593</v>
       </c>
       <c r="C4" t="n">
-        <v>2592848.951119911</v>
+        <v>2543664.396807859</v>
       </c>
       <c r="D4" t="n">
         <v>-0.001359050893601221</v>
@@ -503,7 +503,7 @@
         <v>20994.80346234865</v>
       </c>
       <c r="C5" t="n">
-        <v>2627321.365441931</v>
+        <v>2577482.893232442</v>
       </c>
       <c r="D5" t="n">
         <v>1.329518802363361</v>
@@ -518,7 +518,7 @@
         <v>20786.65317018869</v>
       </c>
       <c r="C6" t="n">
-        <v>2601273.123990393</v>
+        <v>2551928.768935647</v>
       </c>
       <c r="D6" t="n">
         <v>-0.9914372027023388</v>
@@ -533,7 +533,7 @@
         <v>20835.93518869521</v>
       </c>
       <c r="C7" t="n">
-        <v>2607440.350103582</v>
+        <v>2557979.007027769</v>
       </c>
       <c r="D7" t="n">
         <v>0.2370849126265062</v>
@@ -548,7 +548,7 @@
         <v>20983.87360669911</v>
       </c>
       <c r="C8" t="n">
-        <v>2625953.586823725</v>
+        <v>2576141.06043021</v>
       </c>
       <c r="D8" t="n">
         <v>0.7100157332230905</v>
@@ -563,7 +563,7 @@
         <v>21522.28057779043</v>
       </c>
       <c r="C9" t="n">
-        <v>2693330.647103806</v>
+        <v>2642240.024398779</v>
       </c>
       <c r="D9" t="n">
         <v>2.56581306760939</v>
@@ -578,7 +578,7 @@
         <v>21407.53445731089</v>
       </c>
       <c r="C10" t="n">
-        <v>2678971.144549847</v>
+        <v>2628152.911693428</v>
       </c>
       <c r="D10" t="n">
         <v>-0.5331503790446335</v>
@@ -593,7 +593,7 @@
         <v>21379.55582924151</v>
       </c>
       <c r="C11" t="n">
-        <v>2675469.856841473</v>
+        <v>2624718.04099534</v>
       </c>
       <c r="D11" t="n">
         <v>-0.1306952378153259</v>
@@ -608,7 +608,7 @@
         <v>21652.99850527176</v>
       </c>
       <c r="C12" t="n">
-        <v>2709688.885671454</v>
+        <v>2658287.958475712</v>
       </c>
       <c r="D12" t="n">
         <v>1.278991379494676</v>
@@ -623,7 +623,7 @@
         <v>21635.22984610807</v>
       </c>
       <c r="C13" t="n">
-        <v>2707465.288868572</v>
+        <v>2656106.541768848</v>
       </c>
       <c r="D13" t="n">
         <v>-0.08206096333200907</v>
@@ -638,7 +638,7 @@
         <v>21075.59881918914</v>
       </c>
       <c r="C14" t="n">
-        <v>2637432.218236348</v>
+        <v>2587401.950130614</v>
       </c>
       <c r="D14" t="n">
         <v>-2.586665502976415</v>
@@ -655,7 +655,7 @@
         <v>21206.46167729885</v>
       </c>
       <c r="C15" t="n">
-        <v>2653808.593641387</v>
+        <v>2603467.677001655</v>
       </c>
       <c r="D15" t="n">
         <v>0.6209211858339225</v>
@@ -672,7 +672,7 @@
         <v>21098.02661221</v>
       </c>
       <c r="C16" t="n">
-        <v>2640238.866076091</v>
+        <v>2590155.35779875</v>
       </c>
       <c r="D16" t="n">
         <v>-0.5113303045973128</v>
@@ -689,7 +689,7 @@
         <v>21090.28634450593</v>
       </c>
       <c r="C17" t="n">
-        <v>2639270.23730328</v>
+        <v>2589205.103244947</v>
       </c>
       <c r="D17" t="n">
         <v>-0.03668716437958963</v>
@@ -706,7 +706,7 @@
         <v>21102.59361526626</v>
       </c>
       <c r="C18" t="n">
-        <v>2640810.387725592</v>
+        <v>2590716.038077179</v>
       </c>
       <c r="D18" t="n">
         <v>0.05835516198922086</v>
@@ -723,7 +723,7 @@
         <v>21017.93618851875</v>
       </c>
       <c r="C19" t="n">
-        <v>2630216.229679008</v>
+        <v>2580322.843893765</v>
       </c>
       <c r="D19" t="n">
         <v>-0.4011707200117454</v>
@@ -740,7 +740,7 @@
         <v>20439.9424606696</v>
       </c>
       <c r="C20" t="n">
-        <v>2557885.222961425</v>
+        <v>2509363.906431049</v>
       </c>
       <c r="D20" t="n">
         <v>-2.750002296442766</v>
@@ -757,7 +757,7 @@
         <v>20284.34672993223</v>
       </c>
       <c r="C21" t="n">
-        <v>2538413.738578587</v>
+        <v>2490261.782662431</v>
       </c>
       <c r="D21" t="n">
         <v>-0.7612337022805948</v>
@@ -774,7 +774,7 @@
         <v>19972.96642111005</v>
       </c>
       <c r="C22" t="n">
-        <v>2499447.137171074</v>
+        <v>2452034.350778255</v>
       </c>
       <c r="D22" t="n">
         <v>-1.535076840126659</v>
@@ -791,7 +791,7 @@
         <v>19077.63514875183</v>
       </c>
       <c r="C23" t="n">
-        <v>2387404.031588608</v>
+        <v>2342116.625546014</v>
       </c>
       <c r="D23" t="n">
         <v>-4.482715554019601</v>
@@ -808,7 +808,7 @@
         <v>19038.06719943404</v>
       </c>
       <c r="C24" t="n">
-        <v>2382452.438742513</v>
+        <v>2337258.96099727</v>
       </c>
       <c r="D24" t="n">
         <v>-0.2074048958860653</v>
@@ -825,7 +825,7 @@
         <v>18778.6825563297</v>
       </c>
       <c r="C25" t="n">
-        <v>2349992.653352394</v>
+        <v>2305414.915323416</v>
       </c>
       <c r="D25" t="n">
         <v>-1.362452608172582</v>
@@ -842,7 +842,7 @@
         <v>18636.98283684802</v>
       </c>
       <c r="C26" t="n">
-        <v>2332260.136773279</v>
+        <v>2288018.772339994</v>
       </c>
       <c r="D26" t="n">
         <v>-0.7545775325645376</v>
@@ -859,7 +859,7 @@
         <v>18649.97170509377</v>
       </c>
       <c r="C27" t="n">
-        <v>2333885.583332765</v>
+        <v>2289613.385300572</v>
       </c>
       <c r="D27" t="n">
         <v>0.06969405058454559</v>
@@ -876,7 +876,7 @@
         <v>18670.22176862934</v>
       </c>
       <c r="C28" t="n">
-        <v>2336419.706820703</v>
+        <v>2292099.438215686</v>
       </c>
       <c r="D28" t="n">
         <v>0.1085795938770451</v>
@@ -893,7 +893,7 @@
         <v>18879.86867167968</v>
       </c>
       <c r="C29" t="n">
-        <v>2362655.236415952</v>
+        <v>2317837.297929423</v>
       </c>
       <c r="D29" t="n">
         <v>1.122894551807629</v>
@@ -910,7 +910,7 @@
         <v>18614.33163875247</v>
       </c>
       <c r="C30" t="n">
-        <v>2329425.531685595</v>
+        <v>2285237.937753606</v>
       </c>
       <c r="D30" t="n">
         <v>-1.406455932214845</v>
@@ -927,7 +927,7 @@
         <v>18632.4441827197</v>
       </c>
       <c r="C31" t="n">
-        <v>2331692.162751371</v>
+        <v>2287461.57239311</v>
       </c>
       <c r="D31" t="n">
         <v>0.09730429391037188</v>
@@ -944,7 +944,7 @@
         <v>18437.86163689328</v>
       </c>
       <c r="C32" t="n">
-        <v>2307341.809536173</v>
+        <v>2263573.128565158</v>
       </c>
       <c r="D32" t="n">
         <v>-1.044321098822243</v>
@@ -961,7 +961,7 @@
         <v>18781.81644641509</v>
       </c>
       <c r="C33" t="n">
-        <v>2350384.833083585</v>
+        <v>2305799.655675896</v>
       </c>
       <c r="D33" t="n">
         <v>1.865481021039739</v>
@@ -978,7 +978,7 @@
         <v>18402.08390631853</v>
       </c>
       <c r="C34" t="n">
-        <v>2302864.530379232</v>
+        <v>2259180.780302386</v>
       </c>
       <c r="D34" t="n">
         <v>-2.021809451604117</v>
@@ -995,7 +995,7 @@
         <v>17928.02575536971</v>
       </c>
       <c r="C35" t="n">
-        <v>2243540.178489805</v>
+        <v>2200981.770406472</v>
       </c>
       <c r="D35" t="n">
         <v>-2.576111234804501</v>
@@ -1012,7 +1012,7 @@
         <v>18252.76905330373</v>
       </c>
       <c r="C36" t="n">
-        <v>2284179.044506161</v>
+        <v>2240849.745194514</v>
       </c>
       <c r="D36" t="n">
         <v>1.811372330479566</v>
@@ -1029,7 +1029,7 @@
         <v>17785.06221089703</v>
       </c>
       <c r="C37" t="n">
-        <v>2225649.504945468</v>
+        <v>2183430.470586254</v>
       </c>
       <c r="D37" t="n">
         <v>-2.562388430165596</v>
@@ -1046,7 +1046,7 @@
         <v>17489.97862718659</v>
       </c>
       <c r="C38" t="n">
-        <v>2188722.300293899</v>
+        <v>2147203.749509709</v>
       </c>
       <c r="D38" t="n">
         <v>-1.659165316439781</v>
@@ -1063,7 +1063,7 @@
         <v>18310.81265252481</v>
       </c>
       <c r="C39" t="n">
-        <v>2291442.708042434</v>
+        <v>2247975.622048864</v>
       </c>
       <c r="D39" t="n">
         <v>4.693167686679223</v>
@@ -1080,7 +1080,7 @@
         <v>19071.00241488707</v>
       </c>
       <c r="C40" t="n">
-        <v>2386574.001270609</v>
+        <v>2341302.340330034</v>
       </c>
       <c r="D40" t="n">
         <v>4.151589428541502</v>
@@ -1097,7 +1097,7 @@
         <v>18613.18304770227</v>
       </c>
       <c r="C41" t="n">
-        <v>2329281.795269498</v>
+        <v>2285096.927918076</v>
       </c>
       <c r="D41" t="n">
         <v>-2.40060463118299</v>
@@ -1114,7 +1114,7 @@
         <v>18365.41993000871</v>
       </c>
       <c r="C42" t="n">
-        <v>2298276.345094544</v>
+        <v>2254679.629724533</v>
       </c>
       <c r="D42" t="n">
         <v>-1.331116322547266</v>
@@ -1131,7 +1131,7 @@
         <v>18118.87064409462</v>
       </c>
       <c r="C43" t="n">
-        <v>2267422.795658932</v>
+        <v>2224411.350818189</v>
       </c>
       <c r="D43" t="n">
         <v>-1.342464734559246</v>
@@ -1148,7 +1148,7 @@
         <v>18126.29785404899</v>
       </c>
       <c r="C44" t="n">
-        <v>2268352.247912855</v>
+        <v>2225323.172004616</v>
       </c>
       <c r="D44" t="n">
         <v>0.04099157226882255</v>
@@ -1165,7 +1165,7 @@
         <v>18415.68317502607</v>
       </c>
       <c r="C45" t="n">
-        <v>2304566.36337299</v>
+        <v>2260850.33069932</v>
       </c>
       <c r="D45" t="n">
         <v>1.596494349299427</v>
@@ -1182,7 +1182,7 @@
         <v>18028.43799026414</v>
       </c>
       <c r="C46" t="n">
-        <v>2256105.916986144</v>
+        <v>2213309.145519831</v>
       </c>
       <c r="D46" t="n">
         <v>-2.102801080369798</v>
@@ -1199,7 +1199,7 @@
         <v>17861.00772400494</v>
       </c>
       <c r="C47" t="n">
-        <v>2235153.440981626</v>
+        <v>2192754.123518012</v>
       </c>
       <c r="D47" t="n">
         <v>-0.9287009021503589</v>
@@ -1216,7 +1216,7 @@
         <v>18004.99642715143</v>
       </c>
       <c r="C48" t="n">
-        <v>2253172.404428341</v>
+        <v>2210431.279669741</v>
       </c>
       <c r="D48" t="n">
         <v>0.8061622578717564</v>
@@ -1233,7 +1233,7 @@
         <v>17673.32639572251</v>
       </c>
       <c r="C49" t="n">
-        <v>2211666.71653692</v>
+        <v>2169712.926019087</v>
       </c>
       <c r="D49" t="n">
         <v>-1.842099956925058</v>
@@ -1250,7 +1250,7 @@
         <v>17329.07366126381</v>
       </c>
       <c r="C50" t="n">
-        <v>2168586.410213635</v>
+        <v>2127449.823360991</v>
       </c>
       <c r="D50" t="n">
         <v>-1.947866104832507</v>
@@ -1267,7 +1267,7 @@
         <v>16961.27664990233</v>
       </c>
       <c r="C51" t="n">
-        <v>2122559.737573965</v>
+        <v>2082296.244921148</v>
       </c>
       <c r="D51" t="n">
         <v>-2.122427421978301</v>
@@ -1284,7 +1284,7 @@
         <v>17384.09246392111</v>
       </c>
       <c r="C52" t="n">
-        <v>2175471.546146523</v>
+        <v>2134204.353019229</v>
       </c>
       <c r="D52" t="n">
         <v>2.492830125621537</v>
@@ -1301,7 +1301,7 @@
         <v>17392.77259027265</v>
       </c>
       <c r="C53" t="n">
-        <v>2176557.790247785</v>
+        <v>2135269.991819912</v>
       </c>
       <c r="D53" t="n">
         <v>0.04993143225369145</v>
@@ -1318,7 +1318,7 @@
         <v>17745.38008682018</v>
       </c>
       <c r="C54" t="n">
-        <v>2220683.624097848</v>
+        <v>2178558.78906951</v>
       </c>
       <c r="D54" t="n">
         <v>2.027321950640193</v>
@@ -1335,7 +1335,7 @@
         <v>17380.02240119473</v>
       </c>
       <c r="C55" t="n">
-        <v>2174962.212359289</v>
+        <v>2133704.680942258</v>
       </c>
       <c r="D55" t="n">
         <v>-2.058889039501643</v>
@@ -1352,7 +1352,7 @@
         <v>17475.74724739142</v>
       </c>
       <c r="C56" t="n">
-        <v>2186941.363965411</v>
+        <v>2145456.596313685</v>
       </c>
       <c r="D56" t="n">
         <v>0.5507751600487554</v>
@@ -1369,7 +1369,7 @@
         <v>17722.19441648814</v>
       </c>
       <c r="C57" t="n">
-        <v>2217782.134348506</v>
+        <v>2175712.338577314</v>
       </c>
       <c r="D57" t="n">
         <v>1.410223926954024</v>
@@ -1386,7 +1386,7 @@
         <v>17700.06007121554</v>
       </c>
       <c r="C58" t="n">
-        <v>2215012.2090025</v>
+        <v>2172994.956802566</v>
       </c>
       <c r="D58" t="n">
         <v>-0.1248961880928379</v>
@@ -1403,7 +1403,7 @@
         <v>17816.13625664337</v>
       </c>
       <c r="C59" t="n">
-        <v>2229538.157889827</v>
+        <v>2187245.358469266</v>
       </c>
       <c r="D59" t="n">
         <v>0.6557954321104065</v>
@@ -1420,7 +1420,7 @@
         <v>17828.97279046107</v>
       </c>
       <c r="C60" t="n">
-        <v>2231144.541089266</v>
+        <v>2188821.269688576</v>
       </c>
       <c r="D60" t="n">
         <v>0.07205004290935513</v>
@@ -1437,7 +1437,7 @@
         <v>17933.11469190527</v>
       </c>
       <c r="C61" t="n">
-        <v>2244177.015681981</v>
+        <v>2201606.527236831</v>
       </c>
       <c r="D61" t="n">
         <v>0.5841161051068688</v>
@@ -1454,7 +1454,7 @@
         <v>17613.27993887966</v>
       </c>
       <c r="C62" t="n">
-        <v>2204152.412377548</v>
+        <v>2162341.163021199</v>
       </c>
       <c r="D62" t="n">
         <v>-1.783486909666521</v>
@@ -1471,7 +1471,7 @@
         <v>17744.25207803162</v>
       </c>
       <c r="C63" t="n">
-        <v>2220542.46337701</v>
+        <v>2178420.306070079</v>
       </c>
       <c r="D63" t="n">
         <v>0.7435988050291886</v>
@@ -1488,7 +1488,7 @@
         <v>17746.72692865762</v>
       </c>
       <c r="C64" t="n">
-        <v>2220852.169916423</v>
+        <v>2178724.137690282</v>
       </c>
       <c r="D64" t="n">
         <v>0.01394733694672912</v>
@@ -1505,7 +1505,7 @@
         <v>17930.51794775763</v>
       </c>
       <c r="C65" t="n">
-        <v>2243852.055203455</v>
+        <v>2201287.731034206</v>
       </c>
       <c r="D65" t="n">
         <v>1.035633330240882</v>
@@ -1522,7 +1522,7 @@
         <v>17910.33251183258</v>
       </c>
       <c r="C66" t="n">
-        <v>2241326.019312157</v>
+        <v>2198809.612299609</v>
       </c>
       <c r="D66" t="n">
         <v>-0.1125758663740539</v>
@@ -1539,7 +1539,7 @@
         <v>17738.33926179085</v>
       </c>
       <c r="C67" t="n">
-        <v>2219802.524636114</v>
+        <v>2177694.403456191</v>
       </c>
       <c r="D67" t="n">
         <v>-0.9603018253742768</v>
@@ -1556,7 +1556,7 @@
         <v>17816.44981424359</v>
       </c>
       <c r="C68" t="n">
-        <v>2229577.396960762</v>
+        <v>2187283.853202119</v>
       </c>
       <c r="D68" t="n">
         <v>0.4403487344555757</v>
@@ -1573,7 +1573,7 @@
         <v>17471.08050262926</v>
       </c>
       <c r="C69" t="n">
-        <v>2186357.360488424</v>
+        <v>2144883.670979418</v>
       </c>
       <c r="D69" t="n">
         <v>-1.938485586158789</v>
@@ -1590,7 +1590,7 @@
         <v>17078.90276223544</v>
       </c>
       <c r="C70" t="n">
-        <v>2137279.646651509</v>
+        <v>2096736.927487182</v>
       </c>
       <c r="D70" t="n">
         <v>-2.244725163591332</v>
@@ -1607,7 +1607,7 @@
         <v>17101.17960408871</v>
       </c>
       <c r="C71" t="n">
-        <v>2140067.404234504</v>
+        <v>2099471.803233698</v>
       </c>
       <c r="D71" t="n">
         <v>0.1304348538275102</v>
@@ -1624,7 +1624,7 @@
         <v>16956.92452459692</v>
       </c>
       <c r="C72" t="n">
-        <v>2122015.106050242</v>
+        <v>2081761.944681377</v>
       </c>
       <c r="D72" t="n">
         <v>-0.8435387665146732</v>
@@ -1641,7 +1641,7 @@
         <v>17067.90377684652</v>
       </c>
       <c r="C73" t="n">
-        <v>2135903.217033469</v>
+        <v>2095386.607788609</v>
       </c>
       <c r="D73" t="n">
         <v>0.6544774796196862</v>
@@ -1658,7 +1658,7 @@
         <v>17114.15911069001</v>
       </c>
       <c r="C74" t="n">
-        <v>2141691.679263686</v>
+        <v>2101065.266887093</v>
       </c>
       <c r="D74" t="n">
         <v>0.2710077022243018</v>
@@ -1675,7 +1675,7 @@
         <v>16756.75635235528</v>
       </c>
       <c r="C75" t="n">
-        <v>2096965.759122319</v>
+        <v>2057187.766568793</v>
       </c>
       <c r="D75" t="n">
         <v>-2.088345422191862</v>
@@ -1692,7 +1692,7 @@
         <v>17037.68297893887</v>
       </c>
       <c r="C76" t="n">
-        <v>2132121.340810343</v>
+        <v>2091676.471146154</v>
       </c>
       <c r="D76" t="n">
         <v>1.676497650716913</v>
@@ -1709,7 +1709,7 @@
         <v>17368.2059016909</v>
       </c>
       <c r="C77" t="n">
-        <v>2173483.4777921</v>
+        <v>2132253.996948782</v>
       </c>
       <c r="D77" t="n">
         <v>1.939952299620828</v>
@@ -1726,7 +1726,7 @@
         <v>17598.09197705579</v>
       </c>
       <c r="C78" t="n">
-        <v>2202251.767931463</v>
+        <v>2160476.572487914</v>
       </c>
       <c r="D78" t="n">
         <v>1.32360289062734</v>
@@ -1743,7 +1743,7 @@
         <v>17341.48431184015</v>
       </c>
       <c r="C79" t="n">
-        <v>2170139.497742019</v>
+        <v>2128973.449891326</v>
       </c>
       <c r="D79" t="n">
         <v>-1.45815617710261</v>
@@ -1760,7 +1760,7 @@
         <v>17697.74536495572</v>
       </c>
       <c r="C80" t="n">
-        <v>2214722.543170569</v>
+        <v>2172710.78573146</v>
       </c>
       <c r="D80" t="n">
         <v>2.054386156969978</v>
@@ -1777,7 +1777,7 @@
         <v>17875.81408513733</v>
       </c>
       <c r="C81" t="n">
-        <v>2237006.331341726</v>
+        <v>2194571.865827351</v>
       </c>
       <c r="D81" t="n">
         <v>1.006166133083886</v>
@@ -1794,7 +1794,7 @@
         <v>16830.22342501274</v>
       </c>
       <c r="C82" t="n">
-        <v>2106159.539383018</v>
+        <v>2066207.147165999</v>
       </c>
       <c r="D82" t="n">
         <v>-5.849191847402002</v>
@@ -1811,7 +1811,7 @@
         <v>16338.68567131188</v>
       </c>
       <c r="C83" t="n">
-        <v>2044647.763645961</v>
+        <v>2005862.207342489</v>
       </c>
       <c r="D83" t="n">
         <v>-2.920565825468135</v>
@@ -1828,7 +1828,7 @@
         <v>16853.3870293834</v>
       </c>
       <c r="C84" t="n">
-        <v>2109058.26776468</v>
+        <v>2069050.888671752</v>
       </c>
       <c r="D84" t="n">
         <v>3.15020050220598</v>
@@ -1845,7 +1845,7 @@
         <v>15876.05113067791</v>
       </c>
       <c r="C85" t="n">
-        <v>1986752.979578138</v>
+        <v>1949065.647353681</v>
       </c>
       <c r="D85" t="n">
         <v>-5.799047378438171</v>
@@ -1862,7 +1862,7 @@
         <v>13707.10599893207</v>
       </c>
       <c r="C86" t="n">
-        <v>1715327.915022206</v>
+        <v>1682789.328860853</v>
       </c>
       <c r="D86" t="n">
         <v>-13.66174191486888</v>
@@ -1879,7 +1879,7 @@
         <v>13029.8002662141</v>
       </c>
       <c r="C87" t="n">
-        <v>1630568.854252834</v>
+        <v>1599638.088950482</v>
       </c>
       <c r="D87" t="n">
         <v>-4.941274494927972</v>
@@ -1896,7 +1896,7 @@
         <v>12827.06652619082</v>
       </c>
       <c r="C88" t="n">
-        <v>1605198.448303841</v>
+        <v>1574748.942084776</v>
       </c>
       <c r="D88" t="n">
         <v>-1.555923620325628</v>
@@ -1913,7 +1913,7 @@
         <v>13175.66436079539</v>
       </c>
       <c r="C89" t="n">
-        <v>1648822.507011791</v>
+        <v>1617545.482520245</v>
       </c>
       <c r="D89" t="n">
         <v>2.717673864813785</v>
@@ -1930,7 +1930,7 @@
         <v>14056.08598087176</v>
       </c>
       <c r="C90" t="n">
-        <v>1758999.796223951</v>
+        <v>1725632.78463043</v>
       </c>
       <c r="D90" t="n">
         <v>6.682180085704759</v>
@@ -1947,7 +1947,7 @@
         <v>14480.14584808611</v>
       </c>
       <c r="C91" t="n">
-        <v>1812067.287489434</v>
+        <v>1777693.622228247</v>
       </c>
       <c r="D91" t="n">
         <v>3.016912871701516</v>
@@ -1964,7 +1964,7 @@
         <v>14691.77773247068</v>
       </c>
       <c r="C92" t="n">
-        <v>1838551.220642201</v>
+        <v>1803675.173455531</v>
       </c>
       <c r="D92" t="n">
         <v>1.461531441774411</v>
@@ -1981,7 +1981,7 @@
         <v>15053.25838697239</v>
       </c>
       <c r="C93" t="n">
-        <v>1883787.454859372</v>
+        <v>1848053.307543974</v>
       </c>
       <c r="D93" t="n">
         <v>2.460428282295557</v>
@@ -1998,7 +1998,7 @@
         <v>14998.46486662703</v>
       </c>
       <c r="C94" t="n">
-        <v>1876930.511094725</v>
+        <v>1841326.435268012</v>
       </c>
       <c r="D94" t="n">
         <v>-0.3639977401356465</v>
@@ -2015,7 +2015,7 @@
         <v>15095.59882969436</v>
       </c>
       <c r="C95" t="n">
-        <v>1889086.001710987</v>
+        <v>1853251.344620315</v>
       </c>
       <c r="D95" t="n">
         <v>0.6476260332713313</v>
@@ -2032,7 +2032,7 @@
         <v>15675.16257280262</v>
       </c>
       <c r="C96" t="n">
-        <v>1961613.482505679</v>
+        <v>1924403.029182557</v>
       </c>
       <c r="D96" t="n">
         <v>3.839289515088384</v>
@@ -2049,7 +2049,7 @@
         <v>15736.9844292766</v>
       </c>
       <c r="C97" t="n">
-        <v>1969349.962852193</v>
+        <v>1931992.753838723</v>
       </c>
       <c r="D97" t="n">
         <v>0.3943937180035606</v>
@@ -2066,7 +2066,7 @@
         <v>15634.60771256072</v>
       </c>
       <c r="C98" t="n">
-        <v>1956538.386138279</v>
+        <v>1919424.203889032</v>
       </c>
       <c r="D98" t="n">
         <v>-0.6505485035965486</v>
@@ -2083,7 +2083,7 @@
         <v>15699.88129767559</v>
       </c>
       <c r="C99" t="n">
-        <v>1964706.821012121</v>
+        <v>1927437.689193396</v>
       </c>
       <c r="D99" t="n">
         <v>0.4174942302034079</v>
@@ -2100,7 +2100,7 @@
         <v>16271.68741876545</v>
       </c>
       <c r="C100" t="n">
-        <v>2036263.501288936</v>
+        <v>1997636.988653274</v>
       </c>
       <c r="D100" t="n">
         <v>3.642104741100893</v>
@@ -2117,7 +2117,7 @@
         <v>16322.98314401091</v>
       </c>
       <c r="C101" t="n">
-        <v>2042682.725700106</v>
+        <v>2003934.444809662</v>
       </c>
       <c r="D101" t="n">
         <v>0.3152452718966359</v>
@@ -2134,7 +2134,7 @@
         <v>16336.71887504575</v>
       </c>
       <c r="C102" t="n">
-        <v>2044401.635795289</v>
+        <v>2005620.748367199</v>
       </c>
       <c r="D102" t="n">
         <v>0.08414963682592536</v>
@@ -2151,7 +2151,7 @@
         <v>16394.09506957673</v>
       </c>
       <c r="C103" t="n">
-        <v>2051581.779302196</v>
+        <v>2012664.689509472</v>
       </c>
       <c r="D103" t="n">
         <v>0.3512100255248951</v>
@@ -2168,7 +2168,7 @@
         <v>16578.67381766281</v>
       </c>
       <c r="C104" t="n">
-        <v>2074680.242182441</v>
+        <v>2035324.99049773</v>
       </c>
       <c r="D104" t="n">
         <v>1.125885553931028</v>
@@ -2185,7 +2185,7 @@
         <v>16740.75055410738</v>
       </c>
       <c r="C105" t="n">
-        <v>2094962.769392833</v>
+        <v>2055222.772171466</v>
       </c>
       <c r="D105" t="n">
         <v>0.9776218425378014</v>
@@ -2202,7 +2202,7 @@
         <v>16645.89021409754</v>
       </c>
       <c r="C106" t="n">
-        <v>2083091.80339461</v>
+        <v>2043576.990201655</v>
       </c>
       <c r="D106" t="n">
         <v>-0.566643291788127</v>
@@ -2219,7 +2219,7 @@
         <v>16536.83400510494</v>
       </c>
       <c r="C107" t="n">
-        <v>2069444.344944512</v>
+        <v>2030188.414615161</v>
       </c>
       <c r="D107" t="n">
         <v>-0.6551539604667478</v>
@@ -2236,7 +2236,7 @@
         <v>16587.56946150717</v>
       </c>
       <c r="C108" t="n">
-        <v>2075793.456467755</v>
+        <v>2036417.087876695</v>
       </c>
       <c r="D108" t="n">
         <v>0.3068027192301148</v>
@@ -2253,7 +2253,7 @@
         <v>16378.34528143021</v>
       </c>
       <c r="C109" t="n">
-        <v>2049610.827062861</v>
+        <v>2010731.124873229</v>
       </c>
       <c r="D109" t="n">
         <v>-1.261331146570188</v>
@@ -2270,7 +2270,7 @@
         <v>16139.58147865633</v>
       </c>
       <c r="C110" t="n">
-        <v>2019731.564727923</v>
+        <v>1981418.651513977</v>
       </c>
       <c r="D110" t="n">
         <v>-1.457801741697295</v>
@@ -2287,7 +2287,7 @@
         <v>15810.42595388822</v>
       </c>
       <c r="C111" t="n">
-        <v>1978540.54599191</v>
+        <v>1941008.997962124</v>
       </c>
       <c r="D111" t="n">
         <v>-2.039430360715344</v>
@@ -2304,7 +2304,7 @@
         <v>16186.82034197089</v>
       </c>
       <c r="C112" t="n">
-        <v>2025643.107319312</v>
+        <v>1987218.056224165</v>
       </c>
       <c r="D112" t="n">
         <v>2.380672027309294</v>
@@ -2321,7 +2321,7 @@
         <v>16030.10177573459</v>
       </c>
       <c r="C113" t="n">
-        <v>2006031.109608904</v>
+        <v>1967978.08456878</v>
       </c>
       <c r="D113" t="n">
         <v>-0.9681862337715508</v>
@@ -2338,7 +2338,7 @@
         <v>16171.73924797782</v>
       </c>
       <c r="C114" t="n">
-        <v>2023755.836474731</v>
+        <v>1985366.585604397</v>
       </c>
       <c r="D114" t="n">
         <v>0.8835718838518858</v>
@@ -2355,7 +2355,7 @@
         <v>15935.77342000556</v>
       </c>
       <c r="C115" t="n">
-        <v>1994226.716925813</v>
+        <v>1956397.61306428</v>
       </c>
       <c r="D115" t="n">
         <v>-1.459124614575813</v>
@@ -2372,7 +2372,7 @@
         <v>16200.00246397675</v>
       </c>
       <c r="C116" t="n">
-        <v>2027292.737945766</v>
+        <v>1988836.39449666</v>
       </c>
       <c r="D116" t="n">
         <v>1.658087354828242</v>
@@ -2389,7 +2389,7 @@
         <v>16114.31498792558</v>
       </c>
       <c r="C117" t="n">
-        <v>2016569.677976008</v>
+        <v>1978316.743570551</v>
       </c>
       <c r="D117" t="n">
         <v>-0.5289349569033375</v>
@@ -2406,7 +2406,7 @@
         <v>16148.53773379732</v>
       </c>
       <c r="C118" t="n">
-        <v>2020852.364002299</v>
+        <v>1982518.19</v>
       </c>
       <c r="D118" t="n">
         <v>0.2123748102068612</v>

</xml_diff>

<commit_message>
RIPTE real a precios del último IPC publicado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012WiZx484kRcrrNZ4YGQ81g
</commit_message>
<xml_diff>
--- a/data/excel/ripte_real.xlsx
+++ b/data/excel/ripte_real.xlsx
@@ -438,7 +438,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>RIPTE real, a precios del último mes disponible</t>
+          <t>RIPTE real, a precios del último IPC publicado</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -460,7 +460,7 @@
         <v>20690.14</v>
       </c>
       <c r="C2" t="n">
-        <v>2540080.0728724</v>
+        <v>2589195.32033112</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
@@ -473,7 +473,7 @@
         <v>20719.61758472386</v>
       </c>
       <c r="C3" t="n">
-        <v>2543698.9669714</v>
+        <v>2592884.189735662</v>
       </c>
       <c r="D3" t="n">
         <v>0.1424716542462345</v>
@@ -488,7 +488,7 @@
         <v>20719.33599457593</v>
       </c>
       <c r="C4" t="n">
-        <v>2543664.396807859</v>
+        <v>2592848.951119911</v>
       </c>
       <c r="D4" t="n">
         <v>-0.001359050893601221</v>
@@ -503,7 +503,7 @@
         <v>20994.80346234865</v>
       </c>
       <c r="C5" t="n">
-        <v>2577482.893232442</v>
+        <v>2627321.365441931</v>
       </c>
       <c r="D5" t="n">
         <v>1.329518802363361</v>
@@ -518,7 +518,7 @@
         <v>20786.65317018869</v>
       </c>
       <c r="C6" t="n">
-        <v>2551928.768935647</v>
+        <v>2601273.123990393</v>
       </c>
       <c r="D6" t="n">
         <v>-0.9914372027023388</v>
@@ -533,7 +533,7 @@
         <v>20835.93518869521</v>
       </c>
       <c r="C7" t="n">
-        <v>2557979.007027769</v>
+        <v>2607440.350103582</v>
       </c>
       <c r="D7" t="n">
         <v>0.2370849126265062</v>
@@ -548,7 +548,7 @@
         <v>20983.87360669911</v>
       </c>
       <c r="C8" t="n">
-        <v>2576141.06043021</v>
+        <v>2625953.586823725</v>
       </c>
       <c r="D8" t="n">
         <v>0.7100157332230905</v>
@@ -563,7 +563,7 @@
         <v>21522.28057779043</v>
       </c>
       <c r="C9" t="n">
-        <v>2642240.024398779</v>
+        <v>2693330.647103806</v>
       </c>
       <c r="D9" t="n">
         <v>2.56581306760939</v>
@@ -578,7 +578,7 @@
         <v>21407.53445731089</v>
       </c>
       <c r="C10" t="n">
-        <v>2628152.911693428</v>
+        <v>2678971.144549847</v>
       </c>
       <c r="D10" t="n">
         <v>-0.5331503790446335</v>
@@ -593,7 +593,7 @@
         <v>21379.55582924151</v>
       </c>
       <c r="C11" t="n">
-        <v>2624718.04099534</v>
+        <v>2675469.856841473</v>
       </c>
       <c r="D11" t="n">
         <v>-0.1306952378153259</v>
@@ -608,7 +608,7 @@
         <v>21652.99850527176</v>
       </c>
       <c r="C12" t="n">
-        <v>2658287.958475712</v>
+        <v>2709688.885671454</v>
       </c>
       <c r="D12" t="n">
         <v>1.278991379494676</v>
@@ -623,7 +623,7 @@
         <v>21635.22984610807</v>
       </c>
       <c r="C13" t="n">
-        <v>2656106.541768848</v>
+        <v>2707465.288868572</v>
       </c>
       <c r="D13" t="n">
         <v>-0.08206096333200907</v>
@@ -638,7 +638,7 @@
         <v>21075.59881918914</v>
       </c>
       <c r="C14" t="n">
-        <v>2587401.950130614</v>
+        <v>2637432.218236348</v>
       </c>
       <c r="D14" t="n">
         <v>-2.586665502976415</v>
@@ -655,7 +655,7 @@
         <v>21206.46167729885</v>
       </c>
       <c r="C15" t="n">
-        <v>2603467.677001655</v>
+        <v>2653808.593641387</v>
       </c>
       <c r="D15" t="n">
         <v>0.6209211858339225</v>
@@ -672,7 +672,7 @@
         <v>21098.02661221</v>
       </c>
       <c r="C16" t="n">
-        <v>2590155.35779875</v>
+        <v>2640238.866076091</v>
       </c>
       <c r="D16" t="n">
         <v>-0.5113303045973128</v>
@@ -689,7 +689,7 @@
         <v>21090.28634450593</v>
       </c>
       <c r="C17" t="n">
-        <v>2589205.103244947</v>
+        <v>2639270.23730328</v>
       </c>
       <c r="D17" t="n">
         <v>-0.03668716437958963</v>
@@ -706,7 +706,7 @@
         <v>21102.59361526626</v>
       </c>
       <c r="C18" t="n">
-        <v>2590716.038077179</v>
+        <v>2640810.387725592</v>
       </c>
       <c r="D18" t="n">
         <v>0.05835516198922086</v>
@@ -723,7 +723,7 @@
         <v>21017.93618851875</v>
       </c>
       <c r="C19" t="n">
-        <v>2580322.843893765</v>
+        <v>2630216.229679008</v>
       </c>
       <c r="D19" t="n">
         <v>-0.4011707200117454</v>
@@ -740,7 +740,7 @@
         <v>20439.9424606696</v>
       </c>
       <c r="C20" t="n">
-        <v>2509363.906431049</v>
+        <v>2557885.222961425</v>
       </c>
       <c r="D20" t="n">
         <v>-2.750002296442766</v>
@@ -757,7 +757,7 @@
         <v>20284.34672993223</v>
       </c>
       <c r="C21" t="n">
-        <v>2490261.782662431</v>
+        <v>2538413.738578587</v>
       </c>
       <c r="D21" t="n">
         <v>-0.7612337022805948</v>
@@ -774,7 +774,7 @@
         <v>19972.96642111005</v>
       </c>
       <c r="C22" t="n">
-        <v>2452034.350778255</v>
+        <v>2499447.137171074</v>
       </c>
       <c r="D22" t="n">
         <v>-1.535076840126659</v>
@@ -791,7 +791,7 @@
         <v>19077.63514875183</v>
       </c>
       <c r="C23" t="n">
-        <v>2342116.625546014</v>
+        <v>2387404.031588608</v>
       </c>
       <c r="D23" t="n">
         <v>-4.482715554019601</v>
@@ -808,7 +808,7 @@
         <v>19038.06719943404</v>
       </c>
       <c r="C24" t="n">
-        <v>2337258.96099727</v>
+        <v>2382452.438742513</v>
       </c>
       <c r="D24" t="n">
         <v>-0.2074048958860653</v>
@@ -825,7 +825,7 @@
         <v>18778.6825563297</v>
       </c>
       <c r="C25" t="n">
-        <v>2305414.915323416</v>
+        <v>2349992.653352394</v>
       </c>
       <c r="D25" t="n">
         <v>-1.362452608172582</v>
@@ -842,7 +842,7 @@
         <v>18636.98283684802</v>
       </c>
       <c r="C26" t="n">
-        <v>2288018.772339994</v>
+        <v>2332260.136773279</v>
       </c>
       <c r="D26" t="n">
         <v>-0.7545775325645376</v>
@@ -859,7 +859,7 @@
         <v>18649.97170509377</v>
       </c>
       <c r="C27" t="n">
-        <v>2289613.385300572</v>
+        <v>2333885.583332765</v>
       </c>
       <c r="D27" t="n">
         <v>0.06969405058454559</v>
@@ -876,7 +876,7 @@
         <v>18670.22176862934</v>
       </c>
       <c r="C28" t="n">
-        <v>2292099.438215686</v>
+        <v>2336419.706820703</v>
       </c>
       <c r="D28" t="n">
         <v>0.1085795938770451</v>
@@ -893,7 +893,7 @@
         <v>18879.86867167968</v>
       </c>
       <c r="C29" t="n">
-        <v>2317837.297929423</v>
+        <v>2362655.236415952</v>
       </c>
       <c r="D29" t="n">
         <v>1.122894551807629</v>
@@ -910,7 +910,7 @@
         <v>18614.33163875247</v>
       </c>
       <c r="C30" t="n">
-        <v>2285237.937753606</v>
+        <v>2329425.531685595</v>
       </c>
       <c r="D30" t="n">
         <v>-1.406455932214845</v>
@@ -927,7 +927,7 @@
         <v>18632.4441827197</v>
       </c>
       <c r="C31" t="n">
-        <v>2287461.57239311</v>
+        <v>2331692.162751371</v>
       </c>
       <c r="D31" t="n">
         <v>0.09730429391037188</v>
@@ -944,7 +944,7 @@
         <v>18437.86163689328</v>
       </c>
       <c r="C32" t="n">
-        <v>2263573.128565158</v>
+        <v>2307341.809536173</v>
       </c>
       <c r="D32" t="n">
         <v>-1.044321098822243</v>
@@ -961,7 +961,7 @@
         <v>18781.81644641509</v>
       </c>
       <c r="C33" t="n">
-        <v>2305799.655675896</v>
+        <v>2350384.833083585</v>
       </c>
       <c r="D33" t="n">
         <v>1.865481021039739</v>
@@ -978,7 +978,7 @@
         <v>18402.08390631853</v>
       </c>
       <c r="C34" t="n">
-        <v>2259180.780302386</v>
+        <v>2302864.530379232</v>
       </c>
       <c r="D34" t="n">
         <v>-2.021809451604117</v>
@@ -995,7 +995,7 @@
         <v>17928.02575536971</v>
       </c>
       <c r="C35" t="n">
-        <v>2200981.770406472</v>
+        <v>2243540.178489805</v>
       </c>
       <c r="D35" t="n">
         <v>-2.576111234804501</v>
@@ -1012,7 +1012,7 @@
         <v>18252.76905330373</v>
       </c>
       <c r="C36" t="n">
-        <v>2240849.745194514</v>
+        <v>2284179.044506161</v>
       </c>
       <c r="D36" t="n">
         <v>1.811372330479566</v>
@@ -1029,7 +1029,7 @@
         <v>17785.06221089703</v>
       </c>
       <c r="C37" t="n">
-        <v>2183430.470586254</v>
+        <v>2225649.504945468</v>
       </c>
       <c r="D37" t="n">
         <v>-2.562388430165596</v>
@@ -1046,7 +1046,7 @@
         <v>17489.97862718659</v>
       </c>
       <c r="C38" t="n">
-        <v>2147203.749509709</v>
+        <v>2188722.300293899</v>
       </c>
       <c r="D38" t="n">
         <v>-1.659165316439781</v>
@@ -1063,7 +1063,7 @@
         <v>18310.81265252481</v>
       </c>
       <c r="C39" t="n">
-        <v>2247975.622048864</v>
+        <v>2291442.708042434</v>
       </c>
       <c r="D39" t="n">
         <v>4.693167686679223</v>
@@ -1080,7 +1080,7 @@
         <v>19071.00241488707</v>
       </c>
       <c r="C40" t="n">
-        <v>2341302.340330034</v>
+        <v>2386574.001270609</v>
       </c>
       <c r="D40" t="n">
         <v>4.151589428541502</v>
@@ -1097,7 +1097,7 @@
         <v>18613.18304770227</v>
       </c>
       <c r="C41" t="n">
-        <v>2285096.927918076</v>
+        <v>2329281.795269498</v>
       </c>
       <c r="D41" t="n">
         <v>-2.40060463118299</v>
@@ -1114,7 +1114,7 @@
         <v>18365.41993000871</v>
       </c>
       <c r="C42" t="n">
-        <v>2254679.629724533</v>
+        <v>2298276.345094544</v>
       </c>
       <c r="D42" t="n">
         <v>-1.331116322547266</v>
@@ -1131,7 +1131,7 @@
         <v>18118.87064409462</v>
       </c>
       <c r="C43" t="n">
-        <v>2224411.350818189</v>
+        <v>2267422.795658932</v>
       </c>
       <c r="D43" t="n">
         <v>-1.342464734559246</v>
@@ -1148,7 +1148,7 @@
         <v>18126.29785404899</v>
       </c>
       <c r="C44" t="n">
-        <v>2225323.172004616</v>
+        <v>2268352.247912855</v>
       </c>
       <c r="D44" t="n">
         <v>0.04099157226882255</v>
@@ -1165,7 +1165,7 @@
         <v>18415.68317502607</v>
       </c>
       <c r="C45" t="n">
-        <v>2260850.33069932</v>
+        <v>2304566.36337299</v>
       </c>
       <c r="D45" t="n">
         <v>1.596494349299427</v>
@@ -1182,7 +1182,7 @@
         <v>18028.43799026414</v>
       </c>
       <c r="C46" t="n">
-        <v>2213309.145519831</v>
+        <v>2256105.916986144</v>
       </c>
       <c r="D46" t="n">
         <v>-2.102801080369798</v>
@@ -1199,7 +1199,7 @@
         <v>17861.00772400494</v>
       </c>
       <c r="C47" t="n">
-        <v>2192754.123518012</v>
+        <v>2235153.440981626</v>
       </c>
       <c r="D47" t="n">
         <v>-0.9287009021503589</v>
@@ -1216,7 +1216,7 @@
         <v>18004.99642715143</v>
       </c>
       <c r="C48" t="n">
-        <v>2210431.279669741</v>
+        <v>2253172.404428341</v>
       </c>
       <c r="D48" t="n">
         <v>0.8061622578717564</v>
@@ -1233,7 +1233,7 @@
         <v>17673.32639572251</v>
       </c>
       <c r="C49" t="n">
-        <v>2169712.926019087</v>
+        <v>2211666.71653692</v>
       </c>
       <c r="D49" t="n">
         <v>-1.842099956925058</v>
@@ -1250,7 +1250,7 @@
         <v>17329.07366126381</v>
       </c>
       <c r="C50" t="n">
-        <v>2127449.823360991</v>
+        <v>2168586.410213635</v>
       </c>
       <c r="D50" t="n">
         <v>-1.947866104832507</v>
@@ -1267,7 +1267,7 @@
         <v>16961.27664990233</v>
       </c>
       <c r="C51" t="n">
-        <v>2082296.244921148</v>
+        <v>2122559.737573965</v>
       </c>
       <c r="D51" t="n">
         <v>-2.122427421978301</v>
@@ -1284,7 +1284,7 @@
         <v>17384.09246392111</v>
       </c>
       <c r="C52" t="n">
-        <v>2134204.353019229</v>
+        <v>2175471.546146523</v>
       </c>
       <c r="D52" t="n">
         <v>2.492830125621537</v>
@@ -1301,7 +1301,7 @@
         <v>17392.77259027265</v>
       </c>
       <c r="C53" t="n">
-        <v>2135269.991819912</v>
+        <v>2176557.790247785</v>
       </c>
       <c r="D53" t="n">
         <v>0.04993143225369145</v>
@@ -1318,7 +1318,7 @@
         <v>17745.38008682018</v>
       </c>
       <c r="C54" t="n">
-        <v>2178558.78906951</v>
+        <v>2220683.624097848</v>
       </c>
       <c r="D54" t="n">
         <v>2.027321950640193</v>
@@ -1335,7 +1335,7 @@
         <v>17380.02240119473</v>
       </c>
       <c r="C55" t="n">
-        <v>2133704.680942258</v>
+        <v>2174962.212359289</v>
       </c>
       <c r="D55" t="n">
         <v>-2.058889039501643</v>
@@ -1352,7 +1352,7 @@
         <v>17475.74724739142</v>
       </c>
       <c r="C56" t="n">
-        <v>2145456.596313685</v>
+        <v>2186941.363965411</v>
       </c>
       <c r="D56" t="n">
         <v>0.5507751600487554</v>
@@ -1369,7 +1369,7 @@
         <v>17722.19441648814</v>
       </c>
       <c r="C57" t="n">
-        <v>2175712.338577314</v>
+        <v>2217782.134348506</v>
       </c>
       <c r="D57" t="n">
         <v>1.410223926954024</v>
@@ -1386,7 +1386,7 @@
         <v>17700.06007121554</v>
       </c>
       <c r="C58" t="n">
-        <v>2172994.956802566</v>
+        <v>2215012.2090025</v>
       </c>
       <c r="D58" t="n">
         <v>-0.1248961880928379</v>
@@ -1403,7 +1403,7 @@
         <v>17816.13625664337</v>
       </c>
       <c r="C59" t="n">
-        <v>2187245.358469266</v>
+        <v>2229538.157889827</v>
       </c>
       <c r="D59" t="n">
         <v>0.6557954321104065</v>
@@ -1420,7 +1420,7 @@
         <v>17828.97279046107</v>
       </c>
       <c r="C60" t="n">
-        <v>2188821.269688576</v>
+        <v>2231144.541089266</v>
       </c>
       <c r="D60" t="n">
         <v>0.07205004290935513</v>
@@ -1437,7 +1437,7 @@
         <v>17933.11469190527</v>
       </c>
       <c r="C61" t="n">
-        <v>2201606.527236831</v>
+        <v>2244177.015681981</v>
       </c>
       <c r="D61" t="n">
         <v>0.5841161051068688</v>
@@ -1454,7 +1454,7 @@
         <v>17613.27993887966</v>
       </c>
       <c r="C62" t="n">
-        <v>2162341.163021199</v>
+        <v>2204152.412377548</v>
       </c>
       <c r="D62" t="n">
         <v>-1.783486909666521</v>
@@ -1471,7 +1471,7 @@
         <v>17744.25207803162</v>
       </c>
       <c r="C63" t="n">
-        <v>2178420.306070079</v>
+        <v>2220542.46337701</v>
       </c>
       <c r="D63" t="n">
         <v>0.7435988050291886</v>
@@ -1488,7 +1488,7 @@
         <v>17746.72692865762</v>
       </c>
       <c r="C64" t="n">
-        <v>2178724.137690282</v>
+        <v>2220852.169916423</v>
       </c>
       <c r="D64" t="n">
         <v>0.01394733694672912</v>
@@ -1505,7 +1505,7 @@
         <v>17930.51794775763</v>
       </c>
       <c r="C65" t="n">
-        <v>2201287.731034206</v>
+        <v>2243852.055203455</v>
       </c>
       <c r="D65" t="n">
         <v>1.035633330240882</v>
@@ -1522,7 +1522,7 @@
         <v>17910.33251183258</v>
       </c>
       <c r="C66" t="n">
-        <v>2198809.612299609</v>
+        <v>2241326.019312157</v>
       </c>
       <c r="D66" t="n">
         <v>-0.1125758663740539</v>
@@ -1539,7 +1539,7 @@
         <v>17738.33926179085</v>
       </c>
       <c r="C67" t="n">
-        <v>2177694.403456191</v>
+        <v>2219802.524636114</v>
       </c>
       <c r="D67" t="n">
         <v>-0.9603018253742768</v>
@@ -1556,7 +1556,7 @@
         <v>17816.44981424359</v>
       </c>
       <c r="C68" t="n">
-        <v>2187283.853202119</v>
+        <v>2229577.396960762</v>
       </c>
       <c r="D68" t="n">
         <v>0.4403487344555757</v>
@@ -1573,7 +1573,7 @@
         <v>17471.08050262926</v>
       </c>
       <c r="C69" t="n">
-        <v>2144883.670979418</v>
+        <v>2186357.360488424</v>
       </c>
       <c r="D69" t="n">
         <v>-1.938485586158789</v>
@@ -1590,7 +1590,7 @@
         <v>17078.90276223544</v>
       </c>
       <c r="C70" t="n">
-        <v>2096736.927487182</v>
+        <v>2137279.646651509</v>
       </c>
       <c r="D70" t="n">
         <v>-2.244725163591332</v>
@@ -1607,7 +1607,7 @@
         <v>17101.17960408871</v>
       </c>
       <c r="C71" t="n">
-        <v>2099471.803233698</v>
+        <v>2140067.404234504</v>
       </c>
       <c r="D71" t="n">
         <v>0.1304348538275102</v>
@@ -1624,7 +1624,7 @@
         <v>16956.92452459692</v>
       </c>
       <c r="C72" t="n">
-        <v>2081761.944681377</v>
+        <v>2122015.106050242</v>
       </c>
       <c r="D72" t="n">
         <v>-0.8435387665146732</v>
@@ -1641,7 +1641,7 @@
         <v>17067.90377684652</v>
       </c>
       <c r="C73" t="n">
-        <v>2095386.607788609</v>
+        <v>2135903.217033469</v>
       </c>
       <c r="D73" t="n">
         <v>0.6544774796196862</v>
@@ -1658,7 +1658,7 @@
         <v>17114.15911069001</v>
       </c>
       <c r="C74" t="n">
-        <v>2101065.266887093</v>
+        <v>2141691.679263686</v>
       </c>
       <c r="D74" t="n">
         <v>0.2710077022243018</v>
@@ -1675,7 +1675,7 @@
         <v>16756.75635235528</v>
       </c>
       <c r="C75" t="n">
-        <v>2057187.766568793</v>
+        <v>2096965.759122319</v>
       </c>
       <c r="D75" t="n">
         <v>-2.088345422191862</v>
@@ -1692,7 +1692,7 @@
         <v>17037.68297893887</v>
       </c>
       <c r="C76" t="n">
-        <v>2091676.471146154</v>
+        <v>2132121.340810343</v>
       </c>
       <c r="D76" t="n">
         <v>1.676497650716913</v>
@@ -1709,7 +1709,7 @@
         <v>17368.2059016909</v>
       </c>
       <c r="C77" t="n">
-        <v>2132253.996948782</v>
+        <v>2173483.4777921</v>
       </c>
       <c r="D77" t="n">
         <v>1.939952299620828</v>
@@ -1726,7 +1726,7 @@
         <v>17598.09197705579</v>
       </c>
       <c r="C78" t="n">
-        <v>2160476.572487914</v>
+        <v>2202251.767931463</v>
       </c>
       <c r="D78" t="n">
         <v>1.32360289062734</v>
@@ -1743,7 +1743,7 @@
         <v>17341.48431184015</v>
       </c>
       <c r="C79" t="n">
-        <v>2128973.449891326</v>
+        <v>2170139.497742019</v>
       </c>
       <c r="D79" t="n">
         <v>-1.45815617710261</v>
@@ -1760,7 +1760,7 @@
         <v>17697.74536495572</v>
       </c>
       <c r="C80" t="n">
-        <v>2172710.78573146</v>
+        <v>2214722.543170569</v>
       </c>
       <c r="D80" t="n">
         <v>2.054386156969978</v>
@@ -1777,7 +1777,7 @@
         <v>17875.81408513733</v>
       </c>
       <c r="C81" t="n">
-        <v>2194571.865827351</v>
+        <v>2237006.331341726</v>
       </c>
       <c r="D81" t="n">
         <v>1.006166133083886</v>
@@ -1794,7 +1794,7 @@
         <v>16830.22342501274</v>
       </c>
       <c r="C82" t="n">
-        <v>2066207.147165999</v>
+        <v>2106159.539383018</v>
       </c>
       <c r="D82" t="n">
         <v>-5.849191847402002</v>
@@ -1811,7 +1811,7 @@
         <v>16338.68567131188</v>
       </c>
       <c r="C83" t="n">
-        <v>2005862.207342489</v>
+        <v>2044647.763645961</v>
       </c>
       <c r="D83" t="n">
         <v>-2.920565825468135</v>
@@ -1828,7 +1828,7 @@
         <v>16853.3870293834</v>
       </c>
       <c r="C84" t="n">
-        <v>2069050.888671752</v>
+        <v>2109058.26776468</v>
       </c>
       <c r="D84" t="n">
         <v>3.15020050220598</v>
@@ -1845,7 +1845,7 @@
         <v>15876.05113067791</v>
       </c>
       <c r="C85" t="n">
-        <v>1949065.647353681</v>
+        <v>1986752.979578138</v>
       </c>
       <c r="D85" t="n">
         <v>-5.799047378438171</v>
@@ -1862,7 +1862,7 @@
         <v>13707.10599893207</v>
       </c>
       <c r="C86" t="n">
-        <v>1682789.328860853</v>
+        <v>1715327.915022206</v>
       </c>
       <c r="D86" t="n">
         <v>-13.66174191486888</v>
@@ -1879,7 +1879,7 @@
         <v>13029.8002662141</v>
       </c>
       <c r="C87" t="n">
-        <v>1599638.088950482</v>
+        <v>1630568.854252834</v>
       </c>
       <c r="D87" t="n">
         <v>-4.941274494927972</v>
@@ -1896,7 +1896,7 @@
         <v>12827.06652619082</v>
       </c>
       <c r="C88" t="n">
-        <v>1574748.942084776</v>
+        <v>1605198.448303841</v>
       </c>
       <c r="D88" t="n">
         <v>-1.555923620325628</v>
@@ -1913,7 +1913,7 @@
         <v>13175.66436079539</v>
       </c>
       <c r="C89" t="n">
-        <v>1617545.482520245</v>
+        <v>1648822.507011791</v>
       </c>
       <c r="D89" t="n">
         <v>2.717673864813785</v>
@@ -1930,7 +1930,7 @@
         <v>14056.08598087176</v>
       </c>
       <c r="C90" t="n">
-        <v>1725632.78463043</v>
+        <v>1758999.796223951</v>
       </c>
       <c r="D90" t="n">
         <v>6.682180085704759</v>
@@ -1947,7 +1947,7 @@
         <v>14480.14584808611</v>
       </c>
       <c r="C91" t="n">
-        <v>1777693.622228247</v>
+        <v>1812067.287489434</v>
       </c>
       <c r="D91" t="n">
         <v>3.016912871701516</v>
@@ -1964,7 +1964,7 @@
         <v>14691.77773247068</v>
       </c>
       <c r="C92" t="n">
-        <v>1803675.173455531</v>
+        <v>1838551.220642201</v>
       </c>
       <c r="D92" t="n">
         <v>1.461531441774411</v>
@@ -1981,7 +1981,7 @@
         <v>15053.25838697239</v>
       </c>
       <c r="C93" t="n">
-        <v>1848053.307543974</v>
+        <v>1883787.454859372</v>
       </c>
       <c r="D93" t="n">
         <v>2.460428282295557</v>
@@ -1998,7 +1998,7 @@
         <v>14998.46486662703</v>
       </c>
       <c r="C94" t="n">
-        <v>1841326.435268012</v>
+        <v>1876930.511094725</v>
       </c>
       <c r="D94" t="n">
         <v>-0.3639977401356465</v>
@@ -2015,7 +2015,7 @@
         <v>15095.59882969436</v>
       </c>
       <c r="C95" t="n">
-        <v>1853251.344620315</v>
+        <v>1889086.001710987</v>
       </c>
       <c r="D95" t="n">
         <v>0.6476260332713313</v>
@@ -2032,7 +2032,7 @@
         <v>15675.16257280262</v>
       </c>
       <c r="C96" t="n">
-        <v>1924403.029182557</v>
+        <v>1961613.482505679</v>
       </c>
       <c r="D96" t="n">
         <v>3.839289515088384</v>
@@ -2049,7 +2049,7 @@
         <v>15736.9844292766</v>
       </c>
       <c r="C97" t="n">
-        <v>1931992.753838723</v>
+        <v>1969349.962852193</v>
       </c>
       <c r="D97" t="n">
         <v>0.3943937180035606</v>
@@ -2066,7 +2066,7 @@
         <v>15634.60771256072</v>
       </c>
       <c r="C98" t="n">
-        <v>1919424.203889032</v>
+        <v>1956538.386138279</v>
       </c>
       <c r="D98" t="n">
         <v>-0.6505485035965486</v>
@@ -2083,7 +2083,7 @@
         <v>15699.88129767559</v>
       </c>
       <c r="C99" t="n">
-        <v>1927437.689193396</v>
+        <v>1964706.821012121</v>
       </c>
       <c r="D99" t="n">
         <v>0.4174942302034079</v>
@@ -2100,7 +2100,7 @@
         <v>16271.68741876545</v>
       </c>
       <c r="C100" t="n">
-        <v>1997636.988653274</v>
+        <v>2036263.501288936</v>
       </c>
       <c r="D100" t="n">
         <v>3.642104741100893</v>
@@ -2117,7 +2117,7 @@
         <v>16322.98314401091</v>
       </c>
       <c r="C101" t="n">
-        <v>2003934.444809662</v>
+        <v>2042682.725700106</v>
       </c>
       <c r="D101" t="n">
         <v>0.3152452718966359</v>
@@ -2134,7 +2134,7 @@
         <v>16336.71887504575</v>
       </c>
       <c r="C102" t="n">
-        <v>2005620.748367199</v>
+        <v>2044401.635795289</v>
       </c>
       <c r="D102" t="n">
         <v>0.08414963682592536</v>
@@ -2151,7 +2151,7 @@
         <v>16394.09506957673</v>
       </c>
       <c r="C103" t="n">
-        <v>2012664.689509472</v>
+        <v>2051581.779302196</v>
       </c>
       <c r="D103" t="n">
         <v>0.3512100255248951</v>
@@ -2168,7 +2168,7 @@
         <v>16578.67381766281</v>
       </c>
       <c r="C104" t="n">
-        <v>2035324.99049773</v>
+        <v>2074680.242182441</v>
       </c>
       <c r="D104" t="n">
         <v>1.125885553931028</v>
@@ -2185,7 +2185,7 @@
         <v>16740.75055410738</v>
       </c>
       <c r="C105" t="n">
-        <v>2055222.772171466</v>
+        <v>2094962.769392833</v>
       </c>
       <c r="D105" t="n">
         <v>0.9776218425378014</v>
@@ -2202,7 +2202,7 @@
         <v>16645.89021409754</v>
       </c>
       <c r="C106" t="n">
-        <v>2043576.990201655</v>
+        <v>2083091.80339461</v>
       </c>
       <c r="D106" t="n">
         <v>-0.566643291788127</v>
@@ -2219,7 +2219,7 @@
         <v>16536.83400510494</v>
       </c>
       <c r="C107" t="n">
-        <v>2030188.414615161</v>
+        <v>2069444.344944512</v>
       </c>
       <c r="D107" t="n">
         <v>-0.6551539604667478</v>
@@ -2236,7 +2236,7 @@
         <v>16587.56946150717</v>
       </c>
       <c r="C108" t="n">
-        <v>2036417.087876695</v>
+        <v>2075793.456467755</v>
       </c>
       <c r="D108" t="n">
         <v>0.3068027192301148</v>
@@ -2253,7 +2253,7 @@
         <v>16378.34528143021</v>
       </c>
       <c r="C109" t="n">
-        <v>2010731.124873229</v>
+        <v>2049610.827062861</v>
       </c>
       <c r="D109" t="n">
         <v>-1.261331146570188</v>
@@ -2270,7 +2270,7 @@
         <v>16139.58147865633</v>
       </c>
       <c r="C110" t="n">
-        <v>1981418.651513977</v>
+        <v>2019731.564727923</v>
       </c>
       <c r="D110" t="n">
         <v>-1.457801741697295</v>
@@ -2287,7 +2287,7 @@
         <v>15810.42595388822</v>
       </c>
       <c r="C111" t="n">
-        <v>1941008.997962124</v>
+        <v>1978540.54599191</v>
       </c>
       <c r="D111" t="n">
         <v>-2.039430360715344</v>
@@ -2304,7 +2304,7 @@
         <v>16186.82034197089</v>
       </c>
       <c r="C112" t="n">
-        <v>1987218.056224165</v>
+        <v>2025643.107319312</v>
       </c>
       <c r="D112" t="n">
         <v>2.380672027309294</v>
@@ -2321,7 +2321,7 @@
         <v>16030.10177573459</v>
       </c>
       <c r="C113" t="n">
-        <v>1967978.08456878</v>
+        <v>2006031.109608904</v>
       </c>
       <c r="D113" t="n">
         <v>-0.9681862337715508</v>
@@ -2338,7 +2338,7 @@
         <v>16171.73924797782</v>
       </c>
       <c r="C114" t="n">
-        <v>1985366.585604397</v>
+        <v>2023755.836474731</v>
       </c>
       <c r="D114" t="n">
         <v>0.8835718838518858</v>
@@ -2355,7 +2355,7 @@
         <v>15935.77342000556</v>
       </c>
       <c r="C115" t="n">
-        <v>1956397.61306428</v>
+        <v>1994226.716925813</v>
       </c>
       <c r="D115" t="n">
         <v>-1.459124614575813</v>
@@ -2372,7 +2372,7 @@
         <v>16200.00246397675</v>
       </c>
       <c r="C116" t="n">
-        <v>1988836.39449666</v>
+        <v>2027292.737945766</v>
       </c>
       <c r="D116" t="n">
         <v>1.658087354828242</v>
@@ -2389,7 +2389,7 @@
         <v>16114.31498792558</v>
       </c>
       <c r="C117" t="n">
-        <v>1978316.743570551</v>
+        <v>2016569.677976008</v>
       </c>
       <c r="D117" t="n">
         <v>-0.5289349569033375</v>
@@ -2406,7 +2406,7 @@
         <v>16148.53773379732</v>
       </c>
       <c r="C118" t="n">
-        <v>1982518.19</v>
+        <v>2020852.364002299</v>
       </c>
       <c r="D118" t="n">
         <v>0.2123748102068612</v>

</xml_diff>